<commit_message>
Direct Write Excel for GRINDING-01 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_GRINDING-01.xlsx
+++ b/FM-MN-07_GRINDING-01.xlsx
@@ -1757,7 +1757,11 @@
       <c r="E6" s="20" t="inlineStr"/>
       <c r="F6" s="20" t="inlineStr"/>
       <c r="G6" s="20" t="inlineStr"/>
-      <c r="H6" s="20" t="inlineStr"/>
+      <c r="H6" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="20" t="inlineStr"/>
       <c r="J6" s="20" t="inlineStr"/>
       <c r="K6" s="20" t="inlineStr"/>
@@ -1798,7 +1802,11 @@
       <c r="E7" s="20" t="inlineStr"/>
       <c r="F7" s="20" t="inlineStr"/>
       <c r="G7" s="20" t="inlineStr"/>
-      <c r="H7" s="20" t="inlineStr"/>
+      <c r="H7" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="20" t="inlineStr"/>
       <c r="J7" s="20" t="inlineStr"/>
       <c r="K7" s="20" t="inlineStr"/>
@@ -1839,7 +1847,11 @@
       <c r="E8" s="20" t="inlineStr"/>
       <c r="F8" s="20" t="inlineStr"/>
       <c r="G8" s="20" t="inlineStr"/>
-      <c r="H8" s="20" t="inlineStr"/>
+      <c r="H8" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="20" t="inlineStr"/>
       <c r="J8" s="20" t="inlineStr"/>
       <c r="K8" s="20" t="inlineStr"/>
@@ -1880,7 +1892,11 @@
       <c r="E9" s="20" t="inlineStr"/>
       <c r="F9" s="20" t="inlineStr"/>
       <c r="G9" s="20" t="inlineStr"/>
-      <c r="H9" s="20" t="inlineStr"/>
+      <c r="H9" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="20" t="inlineStr"/>
       <c r="J9" s="20" t="inlineStr"/>
       <c r="K9" s="20" t="inlineStr"/>
@@ -1921,7 +1937,11 @@
       <c r="E10" s="20" t="inlineStr"/>
       <c r="F10" s="20" t="inlineStr"/>
       <c r="G10" s="20" t="inlineStr"/>
-      <c r="H10" s="20" t="inlineStr"/>
+      <c r="H10" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="20" t="inlineStr"/>
       <c r="J10" s="20" t="inlineStr"/>
       <c r="K10" s="20" t="inlineStr"/>
@@ -1962,7 +1982,11 @@
       <c r="E11" s="20" t="inlineStr"/>
       <c r="F11" s="20" t="inlineStr"/>
       <c r="G11" s="20" t="inlineStr"/>
-      <c r="H11" s="20" t="inlineStr"/>
+      <c r="H11" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="20" t="inlineStr"/>
       <c r="J11" s="20" t="inlineStr"/>
       <c r="K11" s="20" t="inlineStr"/>
@@ -2003,7 +2027,11 @@
       <c r="E12" s="20" t="inlineStr"/>
       <c r="F12" s="20" t="inlineStr"/>
       <c r="G12" s="20" t="inlineStr"/>
-      <c r="H12" s="20" t="inlineStr"/>
+      <c r="H12" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I12" s="20" t="inlineStr"/>
       <c r="J12" s="20" t="inlineStr"/>
       <c r="K12" s="20" t="inlineStr"/>
@@ -2044,7 +2072,11 @@
       <c r="E13" s="20" t="inlineStr"/>
       <c r="F13" s="20" t="inlineStr"/>
       <c r="G13" s="20" t="inlineStr"/>
-      <c r="H13" s="20" t="inlineStr"/>
+      <c r="H13" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I13" s="20" t="inlineStr"/>
       <c r="J13" s="20" t="inlineStr"/>
       <c r="K13" s="20" t="inlineStr"/>
@@ -2085,7 +2117,11 @@
       <c r="E14" s="20" t="inlineStr"/>
       <c r="F14" s="20" t="inlineStr"/>
       <c r="G14" s="20" t="inlineStr"/>
-      <c r="H14" s="20" t="inlineStr"/>
+      <c r="H14" s="29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I14" s="20" t="inlineStr"/>
       <c r="J14" s="20" t="inlineStr"/>
       <c r="K14" s="20" t="inlineStr"/>
@@ -2155,7 +2191,11 @@
       <c r="E16" s="27" t="inlineStr"/>
       <c r="F16" s="27" t="inlineStr"/>
       <c r="G16" s="27" t="inlineStr"/>
-      <c r="H16" s="27" t="inlineStr"/>
+      <c r="H16" s="37" t="inlineStr">
+        <is>
+          <t>ณัช วิกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="I16" s="27" t="inlineStr"/>
       <c r="J16" s="27" t="inlineStr"/>
       <c r="K16" s="27" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for GRINDING-01 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_GRINDING-01.xlsx
+++ b/FM-MN-07_GRINDING-01.xlsx
@@ -1762,7 +1762,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="20" t="inlineStr"/>
+      <c r="I6" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="20" t="inlineStr"/>
       <c r="K6" s="20" t="inlineStr"/>
       <c r="L6" s="20" t="inlineStr"/>
@@ -1807,7 +1811,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="20" t="inlineStr"/>
+      <c r="I7" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="20" t="inlineStr"/>
       <c r="K7" s="20" t="inlineStr"/>
       <c r="L7" s="20" t="inlineStr"/>
@@ -1852,7 +1860,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="20" t="inlineStr"/>
+      <c r="I8" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="20" t="inlineStr"/>
       <c r="K8" s="20" t="inlineStr"/>
       <c r="L8" s="20" t="inlineStr"/>
@@ -1897,7 +1909,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="20" t="inlineStr"/>
+      <c r="I9" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="20" t="inlineStr"/>
       <c r="K9" s="20" t="inlineStr"/>
       <c r="L9" s="20" t="inlineStr"/>
@@ -1942,7 +1958,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="20" t="inlineStr"/>
+      <c r="I10" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="20" t="inlineStr"/>
       <c r="K10" s="20" t="inlineStr"/>
       <c r="L10" s="20" t="inlineStr"/>
@@ -1987,7 +2007,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="20" t="inlineStr"/>
+      <c r="I11" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="20" t="inlineStr"/>
       <c r="K11" s="20" t="inlineStr"/>
       <c r="L11" s="20" t="inlineStr"/>
@@ -2032,7 +2056,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I12" s="20" t="inlineStr"/>
+      <c r="I12" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J12" s="20" t="inlineStr"/>
       <c r="K12" s="20" t="inlineStr"/>
       <c r="L12" s="20" t="inlineStr"/>
@@ -2077,7 +2105,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I13" s="20" t="inlineStr"/>
+      <c r="I13" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J13" s="20" t="inlineStr"/>
       <c r="K13" s="20" t="inlineStr"/>
       <c r="L13" s="20" t="inlineStr"/>
@@ -2122,7 +2154,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="I14" s="20" t="inlineStr"/>
+      <c r="I14" s="29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J14" s="20" t="inlineStr"/>
       <c r="K14" s="20" t="inlineStr"/>
       <c r="L14" s="20" t="inlineStr"/>
@@ -2196,7 +2232,11 @@
           <t>ณัช วิกรัยเจริญ</t>
         </is>
       </c>
-      <c r="I16" s="27" t="inlineStr"/>
+      <c r="I16" s="37" t="inlineStr">
+        <is>
+          <t>ณัช วิกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="J16" s="27" t="inlineStr"/>
       <c r="K16" s="27" t="inlineStr"/>
       <c r="L16" s="27" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for GRINDING-01 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_GRINDING-01.xlsx
+++ b/FM-MN-07_GRINDING-01.xlsx
@@ -1770,7 +1770,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="20" t="inlineStr"/>
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="20" t="inlineStr"/>
       <c r="L6" s="20" t="inlineStr"/>
       <c r="M6" s="20" t="inlineStr"/>
@@ -1819,7 +1823,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="20" t="inlineStr"/>
+      <c r="J7" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="20" t="inlineStr"/>
       <c r="L7" s="20" t="inlineStr"/>
       <c r="M7" s="20" t="inlineStr"/>
@@ -1868,7 +1876,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="20" t="inlineStr"/>
+      <c r="J8" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="20" t="inlineStr"/>
       <c r="L8" s="20" t="inlineStr"/>
       <c r="M8" s="20" t="inlineStr"/>
@@ -1917,7 +1929,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="20" t="inlineStr"/>
+      <c r="J9" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="20" t="inlineStr"/>
       <c r="L9" s="20" t="inlineStr"/>
       <c r="M9" s="20" t="inlineStr"/>
@@ -1966,7 +1982,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="20" t="inlineStr"/>
+      <c r="J10" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="20" t="inlineStr"/>
       <c r="L10" s="20" t="inlineStr"/>
       <c r="M10" s="20" t="inlineStr"/>
@@ -2015,7 +2035,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J11" s="20" t="inlineStr"/>
+      <c r="J11" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K11" s="20" t="inlineStr"/>
       <c r="L11" s="20" t="inlineStr"/>
       <c r="M11" s="20" t="inlineStr"/>
@@ -2064,7 +2088,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J12" s="20" t="inlineStr"/>
+      <c r="J12" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K12" s="20" t="inlineStr"/>
       <c r="L12" s="20" t="inlineStr"/>
       <c r="M12" s="20" t="inlineStr"/>
@@ -2113,7 +2141,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J13" s="20" t="inlineStr"/>
+      <c r="J13" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K13" s="20" t="inlineStr"/>
       <c r="L13" s="20" t="inlineStr"/>
       <c r="M13" s="20" t="inlineStr"/>
@@ -2162,7 +2194,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="J14" s="20" t="inlineStr"/>
+      <c r="J14" s="29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K14" s="20" t="inlineStr"/>
       <c r="L14" s="20" t="inlineStr"/>
       <c r="M14" s="20" t="inlineStr"/>
@@ -2240,7 +2276,11 @@
           <t>ณัช วิกรัยเจริญ</t>
         </is>
       </c>
-      <c r="J16" s="27" t="inlineStr"/>
+      <c r="J16" s="37" t="inlineStr">
+        <is>
+          <t>ณัช วิกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="K16" s="27" t="inlineStr"/>
       <c r="L16" s="27" t="inlineStr"/>
       <c r="M16" s="27" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for GRINDING-01 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_GRINDING-01.xlsx
+++ b/FM-MN-07_GRINDING-01.xlsx
@@ -1776,7 +1776,11 @@
         </is>
       </c>
       <c r="K6" s="20" t="inlineStr"/>
-      <c r="L6" s="20" t="inlineStr"/>
+      <c r="L6" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="20" t="inlineStr"/>
       <c r="N6" s="20" t="inlineStr"/>
       <c r="O6" s="20" t="inlineStr"/>
@@ -1829,7 +1833,11 @@
         </is>
       </c>
       <c r="K7" s="20" t="inlineStr"/>
-      <c r="L7" s="20" t="inlineStr"/>
+      <c r="L7" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="20" t="inlineStr"/>
       <c r="N7" s="20" t="inlineStr"/>
       <c r="O7" s="20" t="inlineStr"/>
@@ -1882,7 +1890,11 @@
         </is>
       </c>
       <c r="K8" s="20" t="inlineStr"/>
-      <c r="L8" s="20" t="inlineStr"/>
+      <c r="L8" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="20" t="inlineStr"/>
       <c r="N8" s="20" t="inlineStr"/>
       <c r="O8" s="20" t="inlineStr"/>
@@ -1935,7 +1947,11 @@
         </is>
       </c>
       <c r="K9" s="20" t="inlineStr"/>
-      <c r="L9" s="20" t="inlineStr"/>
+      <c r="L9" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="20" t="inlineStr"/>
       <c r="N9" s="20" t="inlineStr"/>
       <c r="O9" s="20" t="inlineStr"/>
@@ -1988,7 +2004,11 @@
         </is>
       </c>
       <c r="K10" s="20" t="inlineStr"/>
-      <c r="L10" s="20" t="inlineStr"/>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="20" t="inlineStr"/>
       <c r="N10" s="20" t="inlineStr"/>
       <c r="O10" s="20" t="inlineStr"/>
@@ -2041,7 +2061,11 @@
         </is>
       </c>
       <c r="K11" s="20" t="inlineStr"/>
-      <c r="L11" s="20" t="inlineStr"/>
+      <c r="L11" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M11" s="20" t="inlineStr"/>
       <c r="N11" s="20" t="inlineStr"/>
       <c r="O11" s="20" t="inlineStr"/>
@@ -2094,7 +2118,11 @@
         </is>
       </c>
       <c r="K12" s="20" t="inlineStr"/>
-      <c r="L12" s="20" t="inlineStr"/>
+      <c r="L12" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M12" s="20" t="inlineStr"/>
       <c r="N12" s="20" t="inlineStr"/>
       <c r="O12" s="20" t="inlineStr"/>
@@ -2147,7 +2175,11 @@
         </is>
       </c>
       <c r="K13" s="20" t="inlineStr"/>
-      <c r="L13" s="20" t="inlineStr"/>
+      <c r="L13" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M13" s="20" t="inlineStr"/>
       <c r="N13" s="20" t="inlineStr"/>
       <c r="O13" s="20" t="inlineStr"/>
@@ -2200,7 +2232,11 @@
         </is>
       </c>
       <c r="K14" s="20" t="inlineStr"/>
-      <c r="L14" s="20" t="inlineStr"/>
+      <c r="L14" s="29" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="M14" s="20" t="inlineStr"/>
       <c r="N14" s="20" t="inlineStr"/>
       <c r="O14" s="20" t="inlineStr"/>
@@ -2282,7 +2318,11 @@
         </is>
       </c>
       <c r="K16" s="27" t="inlineStr"/>
-      <c r="L16" s="27" t="inlineStr"/>
+      <c r="L16" s="37" t="inlineStr">
+        <is>
+          <t>ณัช วิกรัยเจริญ</t>
+        </is>
+      </c>
       <c r="M16" s="27" t="inlineStr"/>
       <c r="N16" s="27" t="inlineStr"/>
       <c r="O16" s="27" t="inlineStr"/>

</xml_diff>